<commit_message>
feat(config): 单封头仅跑 path6+path5，无封头跑 path1–4
新增 path6 单封头编号路径，并按封头类型调整运行时跳过矩阵与相关文档。
</commit_message>
<xml_diff>
--- a/docs/protocols/plc_modbus_寄存器地址表_v0.3_patched.xlsx
+++ b/docs/protocols/plc_modbus_寄存器地址表_v0.3_patched.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="339">
   <si>
     <t>方向</t>
   </si>
@@ -1040,9 +1040,6 @@
   </si>
   <si>
     <t>仅供IPC/HMI调试对账；不参与PLC握手与联锁；PLC程序可不接此地址</t>
-  </si>
-  <si>
-    <t>40186</t>
   </si>
   <si>
     <t>WorkpieceHeadType</t>
@@ -5213,26 +5210,26 @@
       <c r="A119" s="16" t="s">
         <v>162</v>
       </c>
-      <c r="B119" s="17" t="s">
-        <v>336</v>
+      <c r="B119" s="17">
+        <v>40186</v>
       </c>
       <c r="C119" s="17">
         <v>185</v>
       </c>
       <c r="D119" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="E119" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F119" s="17" t="s">
+        <v>164</v>
+      </c>
+      <c r="G119" s="17" t="s">
         <v>337</v>
       </c>
-      <c r="E119" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="F119" s="17" t="s">
-        <v>164</v>
-      </c>
-      <c r="G119" s="17" t="s">
+      <c r="H119" s="17" t="s">
         <v>338</v>
-      </c>
-      <c r="H119" s="17" t="s">
-        <v>339</v>
       </c>
     </row>
   </sheetData>

</xml_diff>